<commit_message>
Auto update P2P and organization activities 2026-09-07 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -1160,7 +1160,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1199,7 +1199,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1238,7 +1238,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1277,12 +1277,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1316,7 +1316,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1355,12 +1355,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1394,12 +1394,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1433,7 +1433,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1472,7 +1472,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1511,7 +1511,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1550,12 +1550,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1576,12 +1576,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
@@ -1589,12 +1589,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1615,12 +1615,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -1628,7 +1628,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1659,7 +1659,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
@@ -1667,12 +1671,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1710,12 +1714,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1753,12 +1757,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1796,12 +1800,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -1839,32 +1843,20 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1875,14 +1867,26 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1893,7 +1897,11 @@
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
@@ -2019,7 +2027,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2066,12 +2074,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -2113,12 +2121,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -2129,8 +2137,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2146,16 +2162,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2211,32 +2219,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Hector Morales</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2266,7 +2274,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Hector Morales</t>
+          <t>Mani Rezaeirad</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2321,7 +2329,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Mani Rezaeirad</t>
+          <t>Iván Joseph Aguilar Monteza</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2376,12 +2384,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Iván Joseph Aguilar Monteza</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2431,7 +2439,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2486,7 +2494,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2541,7 +2549,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2596,7 +2604,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2604,24 +2612,24 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I56" t="inlineStr">
         <is>
           <t>✅</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-14 09:30
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:M73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,12 +486,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gene Climich</t>
+          <t>Mahnaz Lonbani</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Carlos Hisamitsu</t>
+          <t>Daniel Sánchez</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,12 +532,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>René Balderrama</t>
+          <t>Gabriella Nogueira Alves</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -555,7 +555,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Falcon facundo</t>
+          <t>Gene Climich</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -601,7 +601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Falcon facundo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -624,12 +624,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>Adrián Lorente</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -647,12 +647,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>César Fuster Pozo</t>
+          <t>Carlos Hisamitsu</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -670,12 +670,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -693,7 +693,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Marc Ponce</t>
+          <t>César Fuster Pozo</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -716,12 +716,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Gabriella Nogueira Alves</t>
+          <t>René Balderrama</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -739,12 +739,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mahnaz Lonbani</t>
+          <t>Marc Ponce</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -762,12 +762,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Daniel Sánchez</t>
+          <t>María del Rocio Páez Díaz</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -785,19 +785,23 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Adrián Lorente</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -878,7 +882,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -920,7 +928,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -951,7 +959,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -982,12 +990,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Danna Vallès</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1013,12 +1021,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1034,7 +1042,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
@@ -1044,12 +1056,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1065,12 +1077,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
@@ -1079,12 +1091,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1100,12 +1112,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -1114,12 +1126,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1324,12 +1336,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1350,12 +1362,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
@@ -1402,12 +1414,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1428,12 +1440,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
@@ -1441,7 +1453,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1480,12 +1492,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1519,12 +1531,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1558,12 +1570,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1597,12 +1609,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1636,7 +1648,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1667,7 +1679,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
@@ -1675,59 +1691,75 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Cristina Navarrete</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Laura Juan</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1738,39 +1770,39 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Cristina Navarrete</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1781,39 +1813,39 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>noel Carrion Matias</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1824,31 +1856,19 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1886,20 +1906,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1910,26 +1942,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Maria Palmer</t>
+          <t>Jaume Puigdollers</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1972,32 +1992,20 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2008,39 +2016,39 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Maria Palmer</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2051,39 +2059,39 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>noel Carrion Matias</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2094,39 +2102,39 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Laura Juan</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2137,14 +2145,26 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2180,19 +2200,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2223,27 +2247,43 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Jaume Puigdollers</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2259,26 +2299,18 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -2320,12 +2352,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -2367,12 +2399,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -2414,7 +2446,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2508,12 +2540,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -2524,16 +2556,8 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2549,13 +2573,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2602,22 +2634,30 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
@@ -2640,16 +2680,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2657,24 +2693,24 @@
           <t>Joan</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2751,7 +2787,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Jordi Calmet</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2806,7 +2842,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2861,32 +2897,32 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2916,12 +2952,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2971,12 +3007,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Juan Carlos Morales</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3026,12 +3062,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3081,7 +3117,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3136,7 +3172,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3191,7 +3227,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3199,24 +3235,24 @@
           <t>Yunier</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3238,116 +3274,6 @@
         </is>
       </c>
       <c r="M73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Alejandro Requena</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Arnau Rosich Giménez</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M75" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-17 09:25
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N74"/>
+  <dimension ref="A1:N71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Maria Palmer</t>
+          <t>Adrián Lorente</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -515,12 +515,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fatemeh keivani</t>
+          <t>René Balderrama</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Daniel Sánchez</t>
+          <t>Carlos Hisamitsu</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -563,7 +563,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>René Balderrama</t>
+          <t>Marc Ponce</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -587,12 +587,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Marc Ponce</t>
+          <t>Daniel Sánchez</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -611,7 +611,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Laura Juan</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -683,12 +683,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>Mahnaz Lonbani</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -731,12 +731,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>María del Rocio Páez Díaz</t>
+          <t>noel Carrion Matias</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jaume Puigdollers</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -779,12 +779,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cristina Navarrete</t>
+          <t>Gabriella Nogueira Alves</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -803,12 +803,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lorena Morón</t>
+          <t>Laura Juan</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -827,12 +827,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Carlos Hisamitsu</t>
+          <t>Maria Palmer</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -851,12 +851,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Adrián Lorente</t>
+          <t>Jaume Puigdollers</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -875,7 +875,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Fatemeh keivani</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -899,7 +899,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mahnaz Lonbani</t>
+          <t>Lorena Morón</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -923,12 +923,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gabriella Nogueira Alves</t>
+          <t>Cristina Navarrete</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -947,19 +947,23 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>noel Carrion Matias</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -971,12 +975,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -999,18 +1003,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1027,12 +1035,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1043,7 +1051,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1055,12 +1067,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Danna Vallès</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1119,7 +1131,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1141,7 +1153,11 @@
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
@@ -1151,12 +1167,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1172,7 +1188,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
@@ -1183,12 +1203,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1204,7 +1224,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
@@ -1215,12 +1239,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1236,7 +1260,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
@@ -1247,12 +1275,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1283,12 +1311,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1319,12 +1347,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1355,12 +1383,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1391,12 +1419,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1427,7 +1455,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Yonadxandi Manriquez Ledezma</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1453,7 +1481,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
@@ -1463,12 +1495,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1489,7 +1521,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -1499,12 +1535,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1525,7 +1561,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
@@ -1535,12 +1575,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1556,7 +1596,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>✅</t>
@@ -1571,7 +1615,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1651,7 +1695,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1682,7 +1726,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
@@ -1691,12 +1739,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1722,7 +1770,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
@@ -1731,12 +1783,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1762,7 +1814,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
@@ -1771,12 +1827,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1802,16 +1858,24 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1848,14 +1912,18 @@
         </is>
       </c>
       <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1892,14 +1960,18 @@
         </is>
       </c>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1936,19 +2008,23 @@
         </is>
       </c>
       <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -1980,14 +2056,18 @@
         </is>
       </c>
       <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2024,19 +2104,23 @@
         </is>
       </c>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -2068,14 +2152,18 @@
         </is>
       </c>
       <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Biel Domènech</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2123,12 +2211,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2171,7 +2259,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2219,12 +2307,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -2267,12 +2355,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -2315,7 +2403,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2363,32 +2451,32 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2405,13 +2493,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2453,18 +2545,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -2501,38 +2597,42 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2549,18 +2649,26 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Violeta Correa</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -2602,37 +2710,41 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2654,17 +2766,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -2706,17 +2822,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr"/>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
@@ -2767,32 +2887,32 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2823,32 +2943,32 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2879,12 +2999,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2935,7 +3055,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2991,7 +3111,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3047,32 +3167,32 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I71" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3095,174 +3215,6 @@
         </is>
       </c>
       <c r="N71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Alejandro Requena</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N72" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Osley Sorio Pacheco</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Marius Lungu</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N74" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-21 09:39
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -491,12 +491,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Adrián Lorente</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -515,7 +515,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>René Balderrama</t>
+          <t>Gene Climich</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -539,7 +539,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Carlos Hisamitsu</t>
+          <t>Mahnaz Lonbani</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -563,7 +563,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Marc Ponce</t>
+          <t>César Fuster Pozo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -587,12 +587,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Daniel Sánchez</t>
+          <t>Marc Ponce</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Daniel Sánchez</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -635,12 +635,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gene Climich</t>
+          <t>noel Carrion Matias</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -659,12 +659,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Falcon facundo</t>
+          <t>Cristina Navarrete</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -683,12 +683,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mahnaz Lonbani</t>
+          <t>Laura Juan</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -707,12 +707,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>César Fuster Pozo</t>
+          <t>Maria Palmer</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -731,7 +731,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>noel Carrion Matias</t>
+          <t>Jaume Puigdollers</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>Fatemeh keivani</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -779,7 +779,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Gabriella Nogueira Alves</t>
+          <t>Carlos Hisamitsu</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -803,12 +803,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Laura Juan</t>
+          <t>Gabriella Nogueira Alves</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -827,12 +827,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Maria Palmer</t>
+          <t>René Balderrama</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -851,12 +851,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jaume Puigdollers</t>
+          <t>Lorena Morón</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -875,7 +875,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fatemeh keivani</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -899,12 +899,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Lorena Morón</t>
+          <t>Falcon facundo</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -923,18 +923,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Cristina Navarrete</t>
+          <t>Adrián Lorente</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
@@ -947,23 +951,23 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -975,23 +979,23 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1035,12 +1039,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1067,7 +1071,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1099,12 +1103,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1131,12 +1135,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1152,12 +1156,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
@@ -1167,12 +1171,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1203,7 +1207,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1239,12 +1243,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1275,12 +1279,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Alejandro Pascual</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1311,12 +1315,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1332,12 +1336,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -1347,12 +1351,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1383,12 +1387,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -1419,7 +1423,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1455,12 +1459,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1481,12 +1485,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
@@ -1495,12 +1499,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1535,12 +1539,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1575,12 +1579,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1615,12 +1619,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -1655,12 +1659,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -1681,12 +1685,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
@@ -1695,7 +1699,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1739,7 +1743,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1783,12 +1787,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1820,19 +1824,23 @@
         </is>
       </c>
       <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1875,12 +1883,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -1923,12 +1931,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -1971,12 +1979,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -2019,7 +2027,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2067,12 +2075,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -2115,12 +2123,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -2163,12 +2171,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -2211,12 +2219,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2259,7 +2267,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2307,12 +2315,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
@@ -2355,32 +2363,32 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2397,18 +2405,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -2445,38 +2457,42 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I58" t="inlineStr">
         <is>
           <t>✅</t>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-22 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,12 +515,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Gene Climich</t>
+          <t>Lorena Morón</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mahnaz Lonbani</t>
+          <t>René Balderrama</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -563,7 +563,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>César Fuster Pozo</t>
+          <t>Marc Ponce</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -587,12 +587,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Marc Ponce</t>
+          <t>Fatemeh keivani</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Daniel Sánchez</t>
+          <t>Jaume Puigdollers</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -635,7 +635,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>noel Carrion Matias</t>
+          <t>Maria Palmer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cristina Navarrete</t>
+          <t>Laura Juan</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -683,7 +683,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Laura Juan</t>
+          <t>Cristina Navarrete</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Maria Palmer</t>
+          <t>noel Carrion Matias</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -731,7 +731,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jaume Puigdollers</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Fatemeh keivani</t>
+          <t>César Fuster Pozo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -779,12 +779,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Carlos Hisamitsu</t>
+          <t>Gene Climich</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -803,12 +803,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gabriella Nogueira Alves</t>
+          <t>Falcon facundo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -827,18 +827,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>René Balderrama</t>
+          <t>Adrián Lorente</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -851,18 +855,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lorena Morón</t>
+          <t>Daniel Sánchez</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -875,18 +883,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Mahnaz Lonbani</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -899,7 +911,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Falcon facundo</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -911,7 +923,11 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -923,7 +939,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Adrián Lorente</t>
+          <t>Gabriella Nogueira Alves</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -951,12 +967,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Carlos Hisamitsu</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -979,23 +995,23 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1007,12 +1023,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1039,7 +1055,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1071,7 +1087,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1103,12 +1119,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1135,12 +1151,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1171,12 +1187,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1207,7 +1223,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1243,12 +1259,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1279,12 +1295,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Alejandro Pascual</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1351,12 +1367,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -1387,7 +1403,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1423,7 +1439,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1450,7 +1466,11 @@
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -1459,12 +1479,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1485,12 +1505,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
@@ -1499,7 +1519,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1539,12 +1559,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1579,7 +1599,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1619,7 +1639,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1659,12 +1679,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -1690,7 +1710,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
@@ -1699,7 +1723,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1743,7 +1767,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1780,7 +1804,11 @@
         </is>
       </c>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
     </row>
@@ -1979,12 +2007,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -2027,12 +2055,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -2075,12 +2103,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -2123,7 +2151,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2171,7 +2199,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2219,12 +2247,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2267,12 +2295,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
@@ -2315,32 +2343,32 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2357,38 +2385,42 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I56" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2415,12 +2447,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -2467,7 +2499,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2519,12 +2551,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -2571,32 +2603,32 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2618,37 +2650,41 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr"/>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Francesca Pani</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2679,7 +2715,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Violeta Correa</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2735,12 +2771,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -2791,32 +2827,32 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2847,32 +2883,32 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2903,12 +2939,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2959,7 +2995,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3015,7 +3051,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3071,32 +3107,32 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I69" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3119,118 +3155,6 @@
         </is>
       </c>
       <c r="N69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Alejandro Requena</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N70" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Biel Domènech</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M71" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N71" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-23 10:50
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -515,12 +515,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lorena Morón</t>
+          <t>René Balderrama</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -539,7 +539,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>René Balderrama</t>
+          <t>Marc Ponce</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -563,12 +563,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Marc Ponce</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -731,12 +731,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Gene Climich</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -779,7 +779,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Gene Climich</t>
+          <t>Falcon facundo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -803,18 +803,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Falcon facundo</t>
+          <t>Adrián Lorente</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -827,12 +831,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Adrián Lorente</t>
+          <t>Daniel Sánchez</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -855,12 +859,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Daniel Sánchez</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -911,23 +915,23 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Gabriella Nogueira Alves</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -939,7 +943,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gabriella Nogueira Alves</t>
+          <t>Carlos Hisamitsu</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -967,7 +971,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Carlos Hisamitsu</t>
+          <t>Lorena Morón</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -995,23 +999,23 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1119,7 +1123,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1140,7 +1144,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr"/>
@@ -1187,7 +1195,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1208,12 +1216,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-09-28 10:04
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N69"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>René Balderrama</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -515,7 +515,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>René Balderrama</t>
+          <t>Marc Ponce</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Marc Ponce</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -563,12 +563,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Gene Climich</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -587,12 +587,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fatemeh keivani</t>
+          <t>Falcon facundo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -611,12 +611,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jaume Puigdollers</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -635,7 +635,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Maria Palmer</t>
+          <t>noel Carrion Matias</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Laura Juan</t>
+          <t>Cristina Navarrete</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -683,7 +683,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Cristina Navarrete</t>
+          <t>Laura Juan</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -707,12 +707,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>noel Carrion Matias</t>
+          <t>César Fuster Pozo</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -731,12 +731,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Gene Climich</t>
+          <t>Jaume Puigdollers</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -755,12 +755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>César Fuster Pozo</t>
+          <t>Fatemeh keivani</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -779,12 +779,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Falcon facundo</t>
+          <t>Maria Palmer</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -803,7 +803,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Adrián Lorente</t>
+          <t>Gabriella Nogueira Alves</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -831,12 +831,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Daniel Sánchez</t>
+          <t>Lorena Morón</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -859,12 +859,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Daniel Sánchez</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -887,7 +887,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mahnaz Lonbani</t>
+          <t>Carlos Hisamitsu</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -915,7 +915,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gabriella Nogueira Alves</t>
+          <t>Mahnaz Lonbani</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -943,7 +943,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Carlos Hisamitsu</t>
+          <t>Adrián Lorente</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -971,12 +971,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Lorena Morón</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1016,7 +1016,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
@@ -1027,12 +1031,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1059,7 +1063,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1091,7 +1095,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1113,7 +1117,11 @@
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -1123,12 +1131,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Arnau Rosich Giménez</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1159,12 +1167,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1195,7 +1203,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1216,12 +1224,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -1231,7 +1239,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1267,7 +1275,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1303,7 +1311,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1324,12 +1332,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -1339,12 +1347,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1360,12 +1368,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -1375,7 +1383,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1411,7 +1419,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1447,12 +1455,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1473,12 +1481,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
@@ -1487,12 +1495,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C36" t="inlineStr"/>
@@ -1527,12 +1535,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Juan Claros</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1567,12 +1575,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Juan Claros</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1607,12 +1615,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1633,12 +1641,12 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
@@ -1647,12 +1655,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -1687,7 +1695,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1731,7 +1739,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1775,12 +1783,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1823,12 +1831,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1871,12 +1879,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1919,12 +1927,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -1967,12 +1975,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -2015,12 +2023,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -2063,7 +2071,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2111,12 +2119,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -2159,12 +2167,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -2207,12 +2215,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C52" t="inlineStr"/>
@@ -2255,12 +2263,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2303,32 +2311,32 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2345,38 +2353,42 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2403,12 +2415,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -2455,7 +2467,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2507,12 +2519,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
@@ -2559,32 +2571,32 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2606,37 +2618,41 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Jorge Aguilar Liévanos</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2667,12 +2683,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Francesca Pani</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -2723,12 +2739,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -2779,7 +2795,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2787,24 +2803,24 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2835,12 +2851,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2891,7 +2907,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2947,7 +2963,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3003,7 +3019,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3059,32 +3075,32 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I68" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3107,62 +3123,6 @@
         </is>
       </c>
       <c r="N68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Biel Domènech</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr"/>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M69" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N69" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-06 10:38
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N68"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,12 +515,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>Fatemeh keivani</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -539,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fatemeh keivani</t>
+          <t>René Balderrama</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -563,7 +563,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>René Balderrama</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -587,12 +587,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Falcon facundo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -611,18 +611,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>noel Carrion Matias</t>
+          <t>Carlos Hisamitsu</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -635,18 +639,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Falcon facundo</t>
+          <t>Jaume Puigdollers</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -659,7 +667,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Laura Juan</t>
+          <t>Maria Palmer</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -670,7 +678,11 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -683,18 +695,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Maria Palmer</t>
+          <t>Gabriella Nogueira Alves</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -707,7 +723,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jaume Puigdollers</t>
+          <t>Laura Juan</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -718,7 +734,11 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -742,12 +762,18 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>10</v>
+      </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
@@ -755,12 +781,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Gabriella Nogueira Alves</t>
+          <t>noel Carrion Matias</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -783,12 +809,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Gene Climich</t>
+          <t>Daniel Sánchez</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -811,12 +837,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Daniel Sánchez</t>
+          <t>Gene Climich</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -839,12 +865,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Carlos Hisamitsu</t>
+          <t>César Fuster Pozo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -867,12 +893,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>César Fuster Pozo</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -883,11 +909,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>9.23</v>
+      </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
@@ -895,12 +927,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mélina Auradon</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -911,7 +943,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -923,28 +959,28 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
@@ -955,28 +991,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Lorena Morón</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
@@ -987,7 +1023,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Lorena Morón</t>
+          <t>Adrián Lorente</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1008,7 +1044,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
@@ -1019,12 +1059,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mahnaz Lonbani</t>
+          <t>Sonia Shah Llois</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1040,7 +1080,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
@@ -1051,7 +1095,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1087,12 +1131,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Arnau Rosich Giménez</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1123,7 +1167,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Adrián Lorente</t>
+          <t>Mahnaz Lonbani</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1159,12 +1203,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1195,7 +1239,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1231,12 +1275,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1267,12 +1311,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Alex Regueira Araujo</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1303,7 +1347,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1329,7 +1373,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
@@ -1339,12 +1387,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1365,7 +1413,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -1375,12 +1427,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Sonia Shah Llois</t>
+          <t>Mélina Auradon</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -1401,9 +1453,15 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+      <c r="K32" t="n">
+        <v>8.5</v>
+      </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
@@ -1451,7 +1509,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Alex Regueira Araujo</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1491,12 +1549,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Leonardo Antonio Ruggiero</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1517,21 +1575,25 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Roser Carrera</t>
+          <t>Júlia Valls Moix</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1575,12 +1637,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Júlia Valls Moix</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
@@ -1619,12 +1681,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Mar Orts</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1663,7 +1725,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mar Orts</t>
+          <t>Roser Carrera</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1707,12 +1769,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Leonardo Antonio Ruggiero</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -1733,19 +1795,23 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="J40" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
@@ -1799,12 +1865,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -1847,7 +1913,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1895,7 +1961,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1943,12 +2009,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1991,12 +2057,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -2039,12 +2105,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -2087,12 +2153,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -2135,32 +2201,32 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2177,38 +2243,42 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2235,12 +2305,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -2287,7 +2357,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Leticia de Cuevillas</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2339,12 +2409,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2391,12 +2461,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
@@ -2443,7 +2513,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2495,7 +2565,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2547,32 +2617,32 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Alejandro Requena</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2594,12 +2664,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Fiammetta Rofrano</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2655,7 +2729,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Valeria Ontaneda</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2711,7 +2785,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Macarena Sanchez Maeso</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2767,7 +2841,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2823,32 +2897,32 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2879,12 +2953,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -2935,12 +3009,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -2991,7 +3065,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2999,24 +3073,24 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3047,12 +3121,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Jorge Aguilar Liévanos</t>
+          <t>Biel Domènech</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C66" t="inlineStr"/>
@@ -3100,118 +3174,6 @@
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Mariela Villca Vizalla</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N67" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Biel Domènech</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr"/>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N68" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-13 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:M65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,20 +469,15 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Test de BigQuery</t>
+          <t>Python 3</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Python 3</t>
+          <t>PBI 1</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
-        <is>
-          <t>PBI 1</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
         <is>
           <t>PBI 2</t>
         </is>
@@ -510,12 +505,11 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>René Balderrama</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -534,23 +528,26 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Marc Ponce</t>
+          <t>Carlos Hisamitsu</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -558,12 +555,11 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>René Balderrama</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -575,30 +571,37 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Falcon facundo</t>
+          <t>Jaume Puigdollers</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -606,17 +609,16 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Carlos Hisamitsu</t>
+          <t>Maria Palmer</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -634,17 +636,16 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gabriella Nogueira Alves</t>
+          <t>Laura Juan</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -662,12 +663,11 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jaume Puigdollers</t>
+          <t>Cristina Navarrete</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -690,12 +690,11 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Maria Palmer</t>
+          <t>noel Carrion Matias</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -718,45 +717,43 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Laura Juan</t>
+          <t>Falcon facundo</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cristina Navarrete</t>
+          <t>Juan Carlos Loaiza Escobar</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -767,21 +764,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="n">
-        <v>10</v>
-      </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>noel Carrion Matias</t>
+          <t>Irina Mihai</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -797,19 +795,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Gene Climich</t>
+          <t>Marc Ponce</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -825,19 +826,22 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>César Fuster Pozo</t>
+          <t>Gene Climich</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -853,56 +857,58 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Juan Carlos Loaiza Escobar</t>
+          <t>Eduardo Vallejo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Irina Mihai</t>
+          <t>Gabriella Nogueira Alves</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yunier</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -921,54 +927,50 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="n">
-        <v>9.23</v>
-      </c>
+      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Eduardo Vallejo</t>
+          <t>Lorena Morón</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Lorena Morón</t>
+          <t>César Fuster Pozo</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -990,17 +992,16 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Daniel Sánchez</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1026,17 +1027,16 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Adrián Lorente</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1062,17 +1062,16 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1098,17 +1097,16 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Daniel Sánchez</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1134,17 +1132,16 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mahnaz Lonbani</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1170,12 +1167,11 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>Mahnaz Lonbani</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1206,17 +1202,16 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Adrián Lorente</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
@@ -1242,12 +1237,11 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1278,17 +1272,16 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Laritza Magan</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1318,17 +1311,16 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Laritza Magan</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1358,7 +1350,6 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1398,7 +1389,6 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1438,7 +1428,6 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1475,12 +1464,9 @@
         </is>
       </c>
       <c r="J32" t="inlineStr"/>
-      <c r="K32" t="n">
-        <v>8.5</v>
-      </c>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1520,7 +1506,6 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1558,13 +1543,12 @@
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1608,7 +1592,6 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1652,7 +1635,6 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1696,7 +1678,6 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1737,14 +1718,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1785,14 +1765,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1833,14 +1812,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1881,14 +1859,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1929,14 +1906,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1977,14 +1953,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2025,14 +2000,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2073,14 +2047,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2121,14 +2094,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2169,14 +2141,13 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2217,18 +2188,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2269,18 +2239,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2321,18 +2290,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2373,18 +2341,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2425,18 +2392,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2477,18 +2443,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2529,18 +2494,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2581,18 +2545,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2633,18 +2596,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N56" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2689,18 +2651,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N57" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2745,18 +2706,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N58" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2801,18 +2761,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N59" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2857,18 +2816,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L60" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N60" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2913,18 +2871,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N61" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -2969,18 +2926,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N62" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -3025,18 +2981,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L63" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N63" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -3081,18 +3036,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N64" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
@@ -3137,18 +3091,17 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="L65" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="N65" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-14 09:20
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M65"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,12 +509,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Desirée Díaz Risquete</t>
+          <t>Lila Carnauba</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Yunier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -532,22 +532,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Carlos Hisamitsu</t>
+          <t>Desirée Díaz Risquete</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -559,23 +555,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>René Balderrama</t>
+          <t>Carlos Hisamitsu</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
@@ -810,7 +806,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Marc Ponce</t>
+          <t>René Balderrama</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -821,17 +817,17 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -841,7 +837,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gene Climich</t>
+          <t>Marc Ponce</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -965,12 +961,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>César Fuster Pozo</t>
+          <t>Adnan Akortal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -986,7 +982,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
@@ -996,7 +996,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Adnan Akortal</t>
+          <t>Adrián Lorente</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1031,7 +1031,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Adrián Lorente</t>
+          <t>Camila da Camara</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1066,12 +1066,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Camila da Camara</t>
+          <t>César Fuster Pozo</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1101,12 +1101,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Daniel Sánchez</t>
+          <t>Mahnaz Lonbani</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1136,12 +1136,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>GINA MARCELA CAICEDO VALENCIA</t>
+          <t>Daniel Sánchez</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1171,12 +1171,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mahnaz Lonbani</t>
+          <t>GINA MARCELA CAICEDO VALENCIA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1206,7 +1206,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Alejandro Pereyra Gutierrez</t>
+          <t>Gene Climich</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1241,12 +1241,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Derian Palma</t>
+          <t>Alejandro Pereyra Gutierrez</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1276,7 +1276,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Xavier Palet Bustillo</t>
+          <t>Derian Palma</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1302,11 +1302,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -1471,7 +1467,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Vanessa Romero</t>
+          <t>Xavier Palet Bustillo</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1502,7 +1498,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
@@ -1682,12 +1682,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Vanessa Romero</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1718,18 +1718,14 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Bonnie Everitt</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1776,7 +1772,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Bonnie Everitt</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1823,7 +1819,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1870,12 +1866,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Eloisa Estefania Thompson</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C42" t="inlineStr"/>
@@ -1917,12 +1913,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Borja Belmonte</t>
+          <t>Eloisa Estefania Thompson</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Alana</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1964,7 +1960,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jessica Beltran</t>
+          <t>Borja Belmonte</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2011,7 +2007,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Jessica Beltran</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2058,12 +2054,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -2105,7 +2101,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2146,7 +2142,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
@@ -2203,12 +2203,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -2458,7 +2458,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Silvia Vilches</t>
+          <t>Francisco José Jiménez Fernández</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2509,32 +2509,32 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Francisco José Jiménez Fernández</t>
+          <t>Marius Lungu</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Yunier</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2555,7 +2555,11 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2780,32 +2784,32 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Marius Lungu</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2835,12 +2839,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Jorge Kundig</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Joan</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -2890,12 +2894,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
@@ -2945,12 +2949,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Osley Sorio Pacheco</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C63" t="inlineStr"/>
@@ -3000,7 +3004,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Mariela Villca Vizalla</t>
+          <t>Osley Sorio Pacheco</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3008,24 +3012,24 @@
           <t>Alana</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I64" t="inlineStr">
         <is>
           <t>✅</t>
@@ -3055,53 +3059,108 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>Mariela Villca Vizalla</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>Biel Domènech</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>Dagoberto</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M65" t="inlineStr">
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
         <is>
           <t>✅</t>
         </is>

</xml_diff>

<commit_message>
Auto update P2P and organization activities 2026-10-21 10:27
</commit_message>
<xml_diff>
--- a/data/p2p_latest.xlsx
+++ b/data/p2p_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M64"/>
+  <dimension ref="A1:M59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1988,32 +1988,32 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Luis Rayón Liranzo</t>
+          <t>Tatiana Lukina</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Joan</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2039,32 +2039,32 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tatiana Lukina</t>
+          <t>Albert Armentano</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2090,12 +2090,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cristina Fornaguera Torner</t>
+          <t>Jordi Montseny</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -2141,12 +2141,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Àlex Barberà Fabra</t>
+          <t>Hugo Nascimento</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Dagoberto</t>
         </is>
       </c>
       <c r="C47" t="inlineStr"/>
@@ -2192,7 +2192,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Natalia Cuenca</t>
+          <t>Luis Rayón Liranzo</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2243,12 +2243,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Albert Armentano</t>
+          <t>Jorge Kundig</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Irene</t>
+          <t>Joan</t>
         </is>
       </c>
       <c r="C49" t="inlineStr"/>
@@ -2289,12 +2289,16 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Irina Andrade</t>
+          <t>Cristina Fornaguera Torner</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2340,17 +2344,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Leidy Massiel Pimentel Santana</t>
+          <t>Àlex Barberà Fabra</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alana</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C51" t="inlineStr"/>
@@ -2391,37 +2399,41 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Jordi Montseny</t>
+          <t>Mariela Villca Vizalla</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2442,17 +2454,21 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Hugo Nascimento</t>
+          <t>Leticia de Cuevillas</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2493,37 +2509,41 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Alejandro Requena</t>
+          <t>Irina Andrade</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+          <t>Irene</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2553,32 +2573,32 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Fiammetta Rofrano</t>
+          <t>Leidy Massiel Pimentel Santana</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+          <t>Alana</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I55" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2608,32 +2628,32 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Valeria Ontaneda</t>
+          <t>Pau Serrano</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I56" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2663,32 +2683,32 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Macarena Sanchez Maeso</t>
+          <t>Silvia Vilches</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
+          <t>Dagoberto</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr">
         <is>
           <t>✅</t>
@@ -2718,7 +2738,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Pau Serrano</t>
+          <t>Alicia Domínguez</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2773,12 +2793,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Alicia Domínguez</t>
+          <t>Natalia Cuenca</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Dagoberto</t>
+          <t>Irene</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -2825,281 +2845,6 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Silvia Vilches</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Dagoberto</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Marius Lungu</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Yunier</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Leticia de Cuevillas</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Irene</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M62" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Mariela Villca Vizalla</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Alana</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M63" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Jorge Kundig</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Joan</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-      <c r="M64" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>